<commit_message>
Adding content to RIAA Response folder.
</commit_message>
<xml_diff>
--- a/RIAAResponse/FlatSweep.xlsx
+++ b/RIAAResponse/FlatSweep.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="28125"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="41660" yWindow="880" windowWidth="25600" windowHeight="18380" tabRatio="500" activeTab="2"/>
+    <workbookView xWindow="41360" yWindow="280" windowWidth="25600" windowHeight="18380" tabRatio="500" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Request Frequencies" sheetId="1" r:id="rId1"/>
@@ -167,7 +167,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="0.00000000"/>
+    <numFmt numFmtId="164" formatCode="0.00000000"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -244,7 +244,7 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -317,7 +317,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
@@ -1956,11 +1955,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="2136512344"/>
-        <c:axId val="2102724936"/>
+        <c:axId val="2093971144"/>
+        <c:axId val="2093974280"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="2136512344"/>
+        <c:axId val="2093971144"/>
         <c:scaling>
           <c:logBase val="10.0"/>
           <c:orientation val="minMax"/>
@@ -1985,14 +1984,14 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2102724936"/>
+        <c:crossAx val="2093974280"/>
         <c:crossesAt val="-35.0"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="10.0"/>
         <c:minorUnit val="10.0"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="2102724936"/>
+        <c:axId val="2093974280"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="140.0"/>
@@ -2015,7 +2014,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2136512344"/>
+        <c:crossAx val="2093971144"/>
         <c:crossesAt val="16.0"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="25.0"/>
@@ -2023,7 +2022,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:txPr>
         <a:bodyPr/>
@@ -2097,10 +2095,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.0631793674095823"/>
+          <c:x val="0.112823751394892"/>
           <c:y val="0.139511074318731"/>
-          <c:w val="0.894320699319365"/>
-          <c:h val="0.731485138654614"/>
+          <c:w val="0.844676316198376"/>
+          <c:h val="0.697607299829544"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -2962,11 +2960,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="-2145514600"/>
-        <c:axId val="-2145511464"/>
+        <c:axId val="2093087304"/>
+        <c:axId val="2093084168"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="-2145514600"/>
+        <c:axId val="2093087304"/>
         <c:scaling>
           <c:logBase val="10.0"/>
           <c:orientation val="minMax"/>
@@ -2977,6 +2975,32 @@
         <c:axPos val="b"/>
         <c:majorGridlines/>
         <c:minorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1400"/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1400"/>
+                  <a:t>Frequency (Hz)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="0.451863006198927"/>
+              <c:y val="0.880030303326697"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
@@ -2991,14 +3015,14 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-2145511464"/>
+        <c:crossAx val="2093084168"/>
         <c:crossesAt val="-0.05"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="10.0"/>
         <c:minorUnit val="10.0"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="-2145511464"/>
+        <c:axId val="2093084168"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="-0.05"/>
@@ -3006,6 +3030,37 @@
         <c:delete val="0"/>
         <c:axPos val="l"/>
         <c:majorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" vert="horz"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1400"/>
+                  <a:t>Degrees</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1400" baseline="0"/>
+                  <a:t> and dB</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US" sz="1400"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="0.0109242665478907"/>
+              <c:y val="0.378730585819857"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
@@ -3020,7 +3075,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-2145514600"/>
+        <c:crossAx val="2093087304"/>
         <c:crossesAt val="16.0"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -3498,11 +3553,11 @@
         <v>1</v>
       </c>
       <c r="C7" s="1">
-        <f>C6*10^(1/_stepsDecade)</f>
+        <f t="shared" ref="C7:C36" si="0">C6*10^(1/_stepsDecade)</f>
         <v>20.142806588706677</v>
       </c>
       <c r="D7" t="str">
-        <f t="shared" ref="D7:D36" si="0">CONCATENATE(",{""requestFreq"": ", C7, "}")</f>
+        <f t="shared" ref="D7:D36" si="1">CONCATENATE(",{""requestFreq"": ", C7, "}")</f>
         <v>,{"requestFreq": 20.1428065887067}</v>
       </c>
     </row>
@@ -3511,11 +3566,11 @@
         <v>2</v>
       </c>
       <c r="C8" s="1">
-        <f>C7*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>25.358291079377818</v>
       </c>
       <c r="D8" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 25.3582910793778}</v>
       </c>
     </row>
@@ -3524,11 +3579,11 @@
         <v>3</v>
       </c>
       <c r="C9" s="1">
-        <f>C8*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>31.924197039502079</v>
       </c>
       <c r="D9" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 31.9241970395021}</v>
       </c>
     </row>
@@ -3537,11 +3592,11 @@
         <v>4</v>
       </c>
       <c r="C10" s="1">
-        <f>C9*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>40.190182904153289</v>
       </c>
       <c r="D10" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 40.1901829041533}</v>
       </c>
     </row>
@@ -3550,11 +3605,11 @@
         <v>5</v>
       </c>
       <c r="C11" s="1">
-        <f>C10*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>50.596442562694079</v>
       </c>
       <c r="D11" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 50.5964425626941}</v>
       </c>
     </row>
@@ -3563,11 +3618,11 @@
         <v>6</v>
       </c>
       <c r="C12" s="1">
-        <f>C11*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>63.697147288559577</v>
       </c>
       <c r="D12" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 63.6971472885596}</v>
       </c>
     </row>
@@ -3576,11 +3631,11 @@
         <v>7</v>
       </c>
       <c r="C13" s="1">
-        <f>C12*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>80.189957380363595</v>
       </c>
       <c r="D13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 80.1899573803636}</v>
       </c>
     </row>
@@ -3589,11 +3644,11 @@
         <v>8</v>
       </c>
       <c r="C14" s="1">
-        <f>C13*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>100.95317511683096</v>
       </c>
       <c r="D14" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 100.953175116831}</v>
       </c>
     </row>
@@ -3602,11 +3657,11 @@
         <v>9</v>
       </c>
       <c r="C15" s="1">
-        <f>C14*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>127.0925175558851</v>
       </c>
       <c r="D15" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 127.092517555885}</v>
       </c>
     </row>
@@ -3615,11 +3670,11 @@
         <v>10</v>
       </c>
       <c r="C16" s="1">
-        <f>C15*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>160.00000000000009</v>
       </c>
       <c r="D16" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 160}</v>
       </c>
     </row>
@@ -3628,11 +3683,11 @@
         <v>11</v>
       </c>
       <c r="C17" s="1">
-        <f>C16*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>201.42806588706688</v>
       </c>
       <c r="D17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 201.428065887067}</v>
       </c>
     </row>
@@ -3641,11 +3696,11 @@
         <v>12</v>
       </c>
       <c r="C18" s="1">
-        <f>C17*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>253.58291079377832</v>
       </c>
       <c r="D18" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 253.582910793778}</v>
       </c>
     </row>
@@ -3654,11 +3709,11 @@
         <v>13</v>
       </c>
       <c r="C19" s="1">
-        <f>C18*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>319.24197039502099</v>
       </c>
       <c r="D19" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 319.241970395021}</v>
       </c>
     </row>
@@ -3667,11 +3722,11 @@
         <v>14</v>
       </c>
       <c r="C20" s="1">
-        <f>C19*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>401.90182904153318</v>
       </c>
       <c r="D20" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 401.901829041533}</v>
       </c>
     </row>
@@ -3680,11 +3735,11 @@
         <v>15</v>
       </c>
       <c r="C21" s="1">
-        <f>C20*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>505.96442562694119</v>
       </c>
       <c r="D21" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 505.964425626941}</v>
       </c>
     </row>
@@ -3693,11 +3748,11 @@
         <v>16</v>
       </c>
       <c r="C22" s="1">
-        <f>C21*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>636.97147288559631</v>
       </c>
       <c r="D22" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 636.971472885596}</v>
       </c>
     </row>
@@ -3706,11 +3761,11 @@
         <v>17</v>
       </c>
       <c r="C23" s="1">
-        <f>C22*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>801.8995738036366</v>
       </c>
       <c r="D23" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 801.899573803637}</v>
       </c>
     </row>
@@ -3719,11 +3774,11 @@
         <v>18</v>
       </c>
       <c r="C24" s="1">
-        <f>C23*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>1009.5317511683104</v>
       </c>
       <c r="D24" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 1009.53175116831}</v>
       </c>
     </row>
@@ -3732,11 +3787,11 @@
         <v>19</v>
       </c>
       <c r="C25" s="1">
-        <f>C24*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>1270.9251755588521</v>
       </c>
       <c r="D25" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 1270.92517555885}</v>
       </c>
     </row>
@@ -3745,11 +3800,11 @@
         <v>20</v>
       </c>
       <c r="C26" s="1">
-        <f>C25*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>1600.0000000000023</v>
       </c>
       <c r="D26" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 1600}</v>
       </c>
     </row>
@@ -3758,11 +3813,11 @@
         <v>21</v>
       </c>
       <c r="C27" s="1">
-        <f>C26*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>2014.2806588706705</v>
       </c>
       <c r="D27" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 2014.28065887067}</v>
       </c>
     </row>
@@ -3771,11 +3826,11 @@
         <v>22</v>
       </c>
       <c r="C28" s="1">
-        <f>C27*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>2535.8291079377855</v>
       </c>
       <c r="D28" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 2535.82910793779}</v>
       </c>
     </row>
@@ -3784,11 +3839,11 @@
         <v>23</v>
       </c>
       <c r="C29" s="1">
-        <f>C28*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>3192.4197039502124</v>
       </c>
       <c r="D29" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 3192.41970395021}</v>
       </c>
     </row>
@@ -3797,11 +3852,11 @@
         <v>24</v>
       </c>
       <c r="C30" s="1">
-        <f>C29*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>4019.0182904153348</v>
       </c>
       <c r="D30" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 4019.01829041533}</v>
       </c>
     </row>
@@ -3810,11 +3865,11 @@
         <v>25</v>
       </c>
       <c r="C31" s="1">
-        <f>C30*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>5059.6442562694156</v>
       </c>
       <c r="D31" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 5059.64425626942}</v>
       </c>
     </row>
@@ -3823,11 +3878,11 @@
         <v>26</v>
       </c>
       <c r="C32" s="1">
-        <f>C31*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>6369.7147288559672</v>
       </c>
       <c r="D32" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 6369.71472885597}</v>
       </c>
     </row>
@@ -3836,11 +3891,11 @@
         <v>27</v>
       </c>
       <c r="C33" s="1">
-        <f>C32*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>8018.9957380363712</v>
       </c>
       <c r="D33" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 8018.99573803637}</v>
       </c>
     </row>
@@ -3849,11 +3904,11 @@
         <v>28</v>
       </c>
       <c r="C34" s="1">
-        <f>C33*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>10095.317511683112</v>
       </c>
       <c r="D34" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 10095.3175116831}</v>
       </c>
     </row>
@@ -3862,11 +3917,11 @@
         <v>29</v>
       </c>
       <c r="C35" s="1">
-        <f>C34*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>12709.25175558853</v>
       </c>
       <c r="D35" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 12709.2517555885}</v>
       </c>
     </row>
@@ -3875,11 +3930,11 @@
         <v>30</v>
       </c>
       <c r="C36" s="1">
-        <f>C35*10^(1/_stepsDecade)</f>
+        <f t="shared" si="0"/>
         <v>16000.000000000033</v>
       </c>
       <c r="D36" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>,{"requestFreq": 16000}</v>
       </c>
     </row>
@@ -8923,19 +8978,19 @@
         <v>16.001450999999999</v>
       </c>
       <c r="J80" s="4" t="str">
-        <f>IMDIV(J13,J44)</f>
+        <f t="shared" ref="J80:M110" si="15">IMDIV(J13,J44)</f>
         <v>0.999836233176375-1.92801510075298E-06i</v>
       </c>
       <c r="K80" s="4" t="str">
-        <f>IMDIV(K13,K44)</f>
+        <f t="shared" si="15"/>
         <v>0.541523644071195+0.0137473810282117i</v>
       </c>
       <c r="L80" s="4" t="str">
-        <f>IMDIV(L13,L44)</f>
+        <f t="shared" si="15"/>
         <v>0.999846114824733-2.75573020878461E-06i</v>
       </c>
       <c r="M80" s="4" t="str">
-        <f>IMDIV(M13,M44)</f>
+        <f t="shared" si="15"/>
         <v>-0.0979640123079009+0.250941426407869i</v>
       </c>
       <c r="N80" s="4">
@@ -8943,15 +8998,15 @@
         <v>-1.4225770288761295E-3</v>
       </c>
       <c r="O80" s="4">
-        <f t="shared" ref="O80:O141" si="15">20*LOG(IMABS(K80))</f>
+        <f t="shared" ref="O80:O110" si="16">20*LOG(IMABS(K80))</f>
         <v>-5.324853516619358</v>
       </c>
       <c r="P80" s="4">
-        <f t="shared" ref="P80:P141" si="16">20*LOG(IMABS(L80))</f>
+        <f t="shared" ref="P80:P110" si="17">20*LOG(IMABS(L80))</f>
         <v>-1.336732470607902E-3</v>
       </c>
       <c r="Q80" s="4">
-        <f t="shared" ref="Q80:Q141" si="17">20*LOG(IMABS(M80))</f>
+        <f t="shared" ref="Q80:Q110" si="18">20*LOG(IMABS(M80))</f>
         <v>-11.392515713028637</v>
       </c>
       <c r="R80" s="4">
@@ -8959,15 +9014,15 @@
         <v>-1.1048522192435104E-4</v>
       </c>
       <c r="S80" s="4">
-        <f t="shared" ref="S80:S141" si="18">DEGREES(IMARGUMENT(K80))</f>
+        <f t="shared" ref="S80:S110" si="19">DEGREES(IMARGUMENT(K80))</f>
         <v>1.4542260086622838</v>
       </c>
       <c r="T80" s="4">
-        <f t="shared" ref="T80:T141" si="19">DEGREES(IMARGUMENT(L80))</f>
+        <f t="shared" ref="T80:T110" si="20">DEGREES(IMARGUMENT(L80))</f>
         <v>-1.5791601137275107E-4</v>
       </c>
       <c r="U80" s="4">
-        <f t="shared" ref="U80:U141" si="20">DEGREES(IMARGUMENT(M80))</f>
+        <f t="shared" ref="U80:U110" si="21">DEGREES(IMARGUMENT(M80))</f>
         <v>111.32497604524723</v>
       </c>
     </row>
@@ -8976,51 +9031,51 @@
         <v>20.143118000000001</v>
       </c>
       <c r="J81" s="4" t="str">
-        <f>IMDIV(J14,J45)</f>
+        <f t="shared" si="15"/>
         <v>0.999826898796676-8.71151809531831E-07i</v>
       </c>
       <c r="K81" s="4" t="str">
-        <f>IMDIV(K14,K45)</f>
+        <f t="shared" si="15"/>
         <v>-1.23581224447804+1.03701258770847i</v>
       </c>
       <c r="L81" s="4" t="str">
-        <f>IMDIV(L14,L45)</f>
+        <f t="shared" si="15"/>
         <v>0.999835562193172-2.0941742642614E-07i</v>
       </c>
       <c r="M81" s="4" t="str">
-        <f>IMDIV(M14,M45)</f>
+        <f t="shared" si="15"/>
         <v>0.271518265613951-1.42862844897446i</v>
       </c>
       <c r="N81" s="4">
-        <f t="shared" ref="N81:N141" si="21">20*LOG(IMABS(J81))</f>
+        <f t="shared" ref="N81:N110" si="22">20*LOG(IMABS(J81))</f>
         <v>-1.5036680921245483E-3</v>
       </c>
       <c r="O81" s="4">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>4.1541193268253851</v>
       </c>
       <c r="P81" s="4">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>-1.428406087443177E-3</v>
       </c>
       <c r="Q81" s="4">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>3.2524905563470679</v>
       </c>
       <c r="R81" s="4">
-        <f t="shared" ref="R81:R141" si="22">DEGREES(IMARGUMENT(J81))</f>
+        <f t="shared" ref="R81:R110" si="23">DEGREES(IMARGUMENT(J81))</f>
         <v>-4.9921963553309222E-5</v>
       </c>
       <c r="S81" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>139.99883042084909</v>
       </c>
       <c r="T81" s="4">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>-1.2000708060822985E-5</v>
       </c>
       <c r="U81" s="4">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>-79.238980411127187</v>
       </c>
     </row>
@@ -9029,51 +9084,51 @@
         <v>25.362767999999999</v>
       </c>
       <c r="J82" s="4" t="str">
-        <f>IMDIV(J15,J46)</f>
+        <f t="shared" si="15"/>
         <v>0.999839641149045-0.0000038702551994903i</v>
       </c>
       <c r="K82" s="4" t="str">
-        <f>IMDIV(K15,K46)</f>
+        <f t="shared" si="15"/>
         <v>0.840073939255204-0.432018535695997i</v>
       </c>
       <c r="L82" s="4" t="str">
-        <f>IMDIV(L15,L46)</f>
+        <f t="shared" si="15"/>
         <v>0.999851004361652-3.06170771301353E-06i</v>
       </c>
       <c r="M82" s="4" t="str">
-        <f>IMDIV(M15,M46)</f>
+        <f t="shared" si="15"/>
         <v>-0.0910993399574976+0.286791288659203i</v>
       </c>
       <c r="N82" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.3929709074069431E-3</v>
+      </c>
+      <c r="O82" s="4">
+        <f t="shared" si="16"/>
+        <v>-0.49457842343367303</v>
+      </c>
+      <c r="P82" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.2942560521710688E-3</v>
+      </c>
+      <c r="Q82" s="4">
+        <f t="shared" si="18"/>
+        <v>-10.431195407034057</v>
+      </c>
+      <c r="R82" s="4">
+        <f t="shared" si="23"/>
+        <v>-2.2178485373255288E-4</v>
+      </c>
+      <c r="S82" s="4">
+        <f t="shared" si="19"/>
+        <v>-27.215060296838878</v>
+      </c>
+      <c r="T82" s="4">
+        <f t="shared" si="20"/>
+        <v>-1.7544907120414007E-4</v>
+      </c>
+      <c r="U82" s="4">
         <f t="shared" si="21"/>
-        <v>-1.3929709074069431E-3</v>
-      </c>
-      <c r="O82" s="4">
-        <f t="shared" si="15"/>
-        <v>-0.49457842343367303</v>
-      </c>
-      <c r="P82" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.2942560521710688E-3</v>
-      </c>
-      <c r="Q82" s="4">
-        <f t="shared" si="17"/>
-        <v>-10.431195407034057</v>
-      </c>
-      <c r="R82" s="4">
-        <f t="shared" si="22"/>
-        <v>-2.2178485373255288E-4</v>
-      </c>
-      <c r="S82" s="4">
-        <f t="shared" si="18"/>
-        <v>-27.215060296838878</v>
-      </c>
-      <c r="T82" s="4">
-        <f t="shared" si="19"/>
-        <v>-1.7544907120414007E-4</v>
-      </c>
-      <c r="U82" s="4">
-        <f t="shared" si="20"/>
         <v>107.62246610947949</v>
       </c>
     </row>
@@ -9082,51 +9137,51 @@
         <v>31.929302</v>
       </c>
       <c r="J83" s="4" t="str">
-        <f>IMDIV(J16,J47)</f>
+        <f t="shared" si="15"/>
         <v>0.999829665360124-2.33856354532412E-06i</v>
       </c>
       <c r="K83" s="4" t="str">
-        <f>IMDIV(K16,K47)</f>
+        <f t="shared" si="15"/>
         <v>-0.0680803130275845+0.297567026378137i</v>
       </c>
       <c r="L83" s="4" t="str">
-        <f>IMDIV(L16,L47)</f>
+        <f t="shared" si="15"/>
         <v>0.999844072203518-1.65372377654488E-06i</v>
       </c>
       <c r="M83" s="4" t="str">
-        <f>IMDIV(M16,M47)</f>
+        <f t="shared" si="15"/>
         <v>0.0956474555826809+0.264669415135763i</v>
       </c>
       <c r="N83" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.4796338797753571E-3</v>
+      </c>
+      <c r="O83" s="4">
+        <f t="shared" si="16"/>
+        <v>-10.306723338356715</v>
+      </c>
+      <c r="P83" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.3544772229386634E-3</v>
+      </c>
+      <c r="Q83" s="4">
+        <f t="shared" si="18"/>
+        <v>-11.012839481894225</v>
+      </c>
+      <c r="R83" s="4">
+        <f t="shared" si="23"/>
+        <v>-1.3401264826615978E-4</v>
+      </c>
+      <c r="S83" s="4">
+        <f t="shared" si="19"/>
+        <v>102.88689383757257</v>
+      </c>
+      <c r="T83" s="4">
+        <f t="shared" si="20"/>
+        <v>-9.4766169556370823E-5</v>
+      </c>
+      <c r="U83" s="4">
         <f t="shared" si="21"/>
-        <v>-1.4796338797753571E-3</v>
-      </c>
-      <c r="O83" s="4">
-        <f t="shared" si="15"/>
-        <v>-10.306723338356715</v>
-      </c>
-      <c r="P83" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.3544772229386634E-3</v>
-      </c>
-      <c r="Q83" s="4">
-        <f t="shared" si="17"/>
-        <v>-11.012839481894225</v>
-      </c>
-      <c r="R83" s="4">
-        <f t="shared" si="22"/>
-        <v>-1.3401264826615978E-4</v>
-      </c>
-      <c r="S83" s="4">
-        <f t="shared" si="18"/>
-        <v>102.88689383757257</v>
-      </c>
-      <c r="T83" s="4">
-        <f t="shared" si="19"/>
-        <v>-9.4766169556370823E-5</v>
-      </c>
-      <c r="U83" s="4">
-        <f t="shared" si="20"/>
         <v>70.13092378972344</v>
       </c>
     </row>
@@ -9135,51 +9190,51 @@
         <v>40.195312000000001</v>
       </c>
       <c r="J84" s="4" t="str">
-        <f>IMDIV(J17,J48)</f>
+        <f t="shared" si="15"/>
         <v>0.999826711154812-3.23633914006388E-06i</v>
       </c>
       <c r="K84" s="4" t="str">
-        <f>IMDIV(K17,K48)</f>
+        <f t="shared" si="15"/>
         <v>-0.686716123109404-0.162178425472896i</v>
       </c>
       <c r="L84" s="4" t="str">
-        <f>IMDIV(L17,L48)</f>
+        <f t="shared" si="15"/>
         <v>0.999835089482824-2.62025844367212E-06i</v>
       </c>
       <c r="M84" s="4" t="str">
-        <f>IMDIV(M17,M48)</f>
+        <f t="shared" si="15"/>
         <v>-0.0728357925197744-0.874888803692768i</v>
       </c>
       <c r="N84" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.5052981687673998E-3</v>
+      </c>
+      <c r="O84" s="4">
+        <f t="shared" si="16"/>
+        <v>-3.0287455549983475</v>
+      </c>
+      <c r="P84" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.4325126439683629E-3</v>
+      </c>
+      <c r="Q84" s="4">
+        <f t="shared" si="18"/>
+        <v>-1.1309465305271147</v>
+      </c>
+      <c r="R84" s="4">
+        <f t="shared" si="23"/>
+        <v>-1.8546071207063339E-4</v>
+      </c>
+      <c r="S84" s="4">
+        <f t="shared" si="19"/>
+        <v>-166.7122001130322</v>
+      </c>
+      <c r="T84" s="4">
+        <f t="shared" si="20"/>
+        <v>-1.5015451211383533E-4</v>
+      </c>
+      <c r="U84" s="4">
         <f t="shared" si="21"/>
-        <v>-1.5052981687673998E-3</v>
-      </c>
-      <c r="O84" s="4">
-        <f t="shared" si="15"/>
-        <v>-3.0287455549983475</v>
-      </c>
-      <c r="P84" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.4325126439683629E-3</v>
-      </c>
-      <c r="Q84" s="4">
-        <f t="shared" si="17"/>
-        <v>-1.1309465305271147</v>
-      </c>
-      <c r="R84" s="4">
-        <f t="shared" si="22"/>
-        <v>-1.8546071207063339E-4</v>
-      </c>
-      <c r="S84" s="4">
-        <f t="shared" si="18"/>
-        <v>-166.7122001130322</v>
-      </c>
-      <c r="T84" s="4">
-        <f t="shared" si="19"/>
-        <v>-1.5015451211383533E-4</v>
-      </c>
-      <c r="U84" s="4">
-        <f t="shared" si="20"/>
         <v>-94.758984463127277</v>
       </c>
     </row>
@@ -9188,51 +9243,51 @@
         <v>50.597405000000002</v>
       </c>
       <c r="J85" s="4" t="str">
-        <f>IMDIV(J18,J49)</f>
+        <f t="shared" si="15"/>
         <v>0.999841771506812-7.15239255033412E-06i</v>
       </c>
       <c r="K85" s="4" t="str">
-        <f>IMDIV(K18,K49)</f>
+        <f t="shared" si="15"/>
         <v>0.364693541368136+1.04555119262915i</v>
       </c>
       <c r="L85" s="4" t="str">
-        <f>IMDIV(L18,L49)</f>
+        <f t="shared" si="15"/>
         <v>0.999853091769855-6.39936539968152E-06i</v>
       </c>
       <c r="M85" s="4" t="str">
-        <f>IMDIV(M18,M49)</f>
+        <f t="shared" si="15"/>
         <v>0.429094912444415+1.18154600625503i</v>
       </c>
       <c r="N85" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.3744637497367148E-3</v>
+      </c>
+      <c r="O85" s="4">
+        <f t="shared" si="16"/>
+        <v>0.88553759040569446</v>
+      </c>
+      <c r="P85" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.2761222347973198E-3</v>
+      </c>
+      <c r="Q85" s="4">
+        <f t="shared" si="18"/>
+        <v>1.9870474919813972</v>
+      </c>
+      <c r="R85" s="4">
+        <f t="shared" si="23"/>
+        <v>-4.0986675914767386E-4</v>
+      </c>
+      <c r="S85" s="4">
+        <f t="shared" si="19"/>
+        <v>70.770970076402477</v>
+      </c>
+      <c r="T85" s="4">
+        <f t="shared" si="20"/>
+        <v>-3.6671050174958135E-4</v>
+      </c>
+      <c r="U85" s="4">
         <f t="shared" si="21"/>
-        <v>-1.3744637497367148E-3</v>
-      </c>
-      <c r="O85" s="4">
-        <f t="shared" si="15"/>
-        <v>0.88553759040569446</v>
-      </c>
-      <c r="P85" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.2761222347973198E-3</v>
-      </c>
-      <c r="Q85" s="4">
-        <f t="shared" si="17"/>
-        <v>1.9870474919813972</v>
-      </c>
-      <c r="R85" s="4">
-        <f t="shared" si="22"/>
-        <v>-4.0986675914767386E-4</v>
-      </c>
-      <c r="S85" s="4">
-        <f t="shared" si="18"/>
-        <v>70.770970076402477</v>
-      </c>
-      <c r="T85" s="4">
-        <f t="shared" si="19"/>
-        <v>-3.6671050174958135E-4</v>
-      </c>
-      <c r="U85" s="4">
-        <f t="shared" si="20"/>
         <v>70.040803364818558</v>
       </c>
     </row>
@@ -9241,51 +9296,51 @@
         <v>63.69847</v>
       </c>
       <c r="J86" s="4" t="str">
-        <f>IMDIV(J19,J50)</f>
+        <f t="shared" si="15"/>
         <v>0.999850994091395-4.99515405393352E-06i</v>
       </c>
       <c r="K86" s="4" t="str">
-        <f>IMDIV(K19,K50)</f>
+        <f t="shared" si="15"/>
         <v>-0.716754503956094-2.91036769079077i</v>
       </c>
       <c r="L86" s="4" t="str">
-        <f>IMDIV(L19,L50)</f>
+        <f t="shared" si="15"/>
         <v>0.999862863187758-3.15519015281598E-06i</v>
       </c>
       <c r="M86" s="4" t="str">
-        <f>IMDIV(M19,M50)</f>
+        <f t="shared" si="15"/>
         <v>-0.0409868440305052-0.376885597288257i</v>
       </c>
       <c r="N86" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.2943452041133357E-3</v>
+      </c>
+      <c r="O86" s="4">
+        <f t="shared" si="16"/>
+        <v>9.5346863694868293</v>
+      </c>
+      <c r="P86" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.1912368562846051E-3</v>
+      </c>
+      <c r="Q86" s="4">
+        <f t="shared" si="18"/>
+        <v>-8.4247470872486154</v>
+      </c>
+      <c r="R86" s="4">
+        <f t="shared" si="23"/>
+        <v>-2.8624389733767865E-4</v>
+      </c>
+      <c r="S86" s="4">
+        <f t="shared" si="19"/>
+        <v>-103.83526451033192</v>
+      </c>
+      <c r="T86" s="4">
+        <f t="shared" si="20"/>
+        <v>-1.8080387418393945E-4</v>
+      </c>
+      <c r="U86" s="4">
         <f t="shared" si="21"/>
-        <v>-1.2943452041133357E-3</v>
-      </c>
-      <c r="O86" s="4">
-        <f t="shared" si="15"/>
-        <v>9.5346863694868293</v>
-      </c>
-      <c r="P86" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.1912368562846051E-3</v>
-      </c>
-      <c r="Q86" s="4">
-        <f t="shared" si="17"/>
-        <v>-8.4247470872486154</v>
-      </c>
-      <c r="R86" s="4">
-        <f t="shared" si="22"/>
-        <v>-2.8624389733767865E-4</v>
-      </c>
-      <c r="S86" s="4">
-        <f t="shared" si="18"/>
-        <v>-103.83526451033192</v>
-      </c>
-      <c r="T86" s="4">
-        <f t="shared" si="19"/>
-        <v>-1.8080387418393945E-4</v>
-      </c>
-      <c r="U86" s="4">
-        <f t="shared" si="20"/>
         <v>-96.206605855671057</v>
       </c>
     </row>
@@ -9294,51 +9349,51 @@
         <v>80.201261000000002</v>
       </c>
       <c r="J87" s="4" t="str">
-        <f>IMDIV(J20,J51)</f>
+        <f t="shared" si="15"/>
         <v>0.999849130623611-5.17404227608061E-06i</v>
       </c>
       <c r="K87" s="4" t="str">
-        <f>IMDIV(K20,K51)</f>
+        <f t="shared" si="15"/>
         <v>0.387692276856272-0.156060824977755i</v>
       </c>
       <c r="L87" s="4" t="str">
-        <f>IMDIV(L20,L51)</f>
+        <f t="shared" si="15"/>
         <v>0.999861267813988-4.30219882823781E-06i</v>
       </c>
       <c r="M87" s="4" t="str">
-        <f>IMDIV(M20,M51)</f>
+        <f t="shared" si="15"/>
         <v>1.30797255706538-0.0170404061315505i</v>
       </c>
       <c r="N87" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.3105334989608778E-3</v>
+      </c>
+      <c r="O87" s="4">
+        <f t="shared" si="16"/>
+        <v>-7.5780584142286038</v>
+      </c>
+      <c r="P87" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.2050959712804274E-3</v>
+      </c>
+      <c r="Q87" s="4">
+        <f t="shared" si="18"/>
+        <v>2.3327097128949643</v>
+      </c>
+      <c r="R87" s="4">
+        <f t="shared" si="23"/>
+        <v>-2.9649551753286734E-4</v>
+      </c>
+      <c r="S87" s="4">
+        <f t="shared" si="19"/>
+        <v>-21.926652684305719</v>
+      </c>
+      <c r="T87" s="4">
+        <f t="shared" si="20"/>
+        <v>-2.4653203741110545E-4</v>
+      </c>
+      <c r="U87" s="4">
         <f t="shared" si="21"/>
-        <v>-1.3105334989608778E-3</v>
-      </c>
-      <c r="O87" s="4">
-        <f t="shared" si="15"/>
-        <v>-7.5780584142286038</v>
-      </c>
-      <c r="P87" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.2050959712804274E-3</v>
-      </c>
-      <c r="Q87" s="4">
-        <f t="shared" si="17"/>
-        <v>2.3327097128949643</v>
-      </c>
-      <c r="R87" s="4">
-        <f t="shared" si="22"/>
-        <v>-2.9649551753286734E-4</v>
-      </c>
-      <c r="S87" s="4">
-        <f t="shared" si="18"/>
-        <v>-21.926652684305719</v>
-      </c>
-      <c r="T87" s="4">
-        <f t="shared" si="19"/>
-        <v>-2.4653203741110545E-4</v>
-      </c>
-      <c r="U87" s="4">
-        <f t="shared" si="20"/>
         <v>-0.7464133051688846</v>
       </c>
     </row>
@@ -9347,51 +9402,51 @@
         <v>100.96802700000001</v>
       </c>
       <c r="J88" s="4" t="str">
-        <f>IMDIV(J21,J52)</f>
+        <f t="shared" si="15"/>
         <v>0.999858462125163-6.43801408912595E-06i</v>
       </c>
       <c r="K88" s="4" t="str">
-        <f>IMDIV(K21,K52)</f>
+        <f t="shared" si="15"/>
         <v>0.357994627570772-0.0693810620159676i</v>
       </c>
       <c r="L88" s="4" t="str">
-        <f>IMDIV(L21,L52)</f>
+        <f t="shared" si="15"/>
         <v>0.999866925233044-5.73508978774563E-06i</v>
       </c>
       <c r="M88" s="4" t="str">
-        <f>IMDIV(M21,M52)</f>
+        <f t="shared" si="15"/>
         <v>-0.0747506117451848-0.0637931844473463i</v>
       </c>
       <c r="N88" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.229469190675896E-3</v>
+      </c>
+      <c r="O88" s="4">
+        <f t="shared" si="16"/>
+        <v>-8.7623364215281008</v>
+      </c>
+      <c r="P88" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.1559495120803925E-3</v>
+      </c>
+      <c r="Q88" s="4">
+        <f t="shared" si="18"/>
+        <v>-20.15147679776652</v>
+      </c>
+      <c r="R88" s="4">
+        <f t="shared" si="23"/>
+        <v>-3.6892325236069729E-4</v>
+      </c>
+      <c r="S88" s="4">
+        <f t="shared" si="19"/>
+        <v>-10.968220520102596</v>
+      </c>
+      <c r="T88" s="4">
+        <f t="shared" si="20"/>
+        <v>-3.2864017367732464E-4</v>
+      </c>
+      <c r="U88" s="4">
         <f t="shared" si="21"/>
-        <v>-1.229469190675896E-3</v>
-      </c>
-      <c r="O88" s="4">
-        <f t="shared" si="15"/>
-        <v>-8.7623364215281008</v>
-      </c>
-      <c r="P88" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.1559495120803925E-3</v>
-      </c>
-      <c r="Q88" s="4">
-        <f t="shared" si="17"/>
-        <v>-20.15147679776652</v>
-      </c>
-      <c r="R88" s="4">
-        <f t="shared" si="22"/>
-        <v>-3.6892325236069729E-4</v>
-      </c>
-      <c r="S88" s="4">
-        <f t="shared" si="18"/>
-        <v>-10.968220520102596</v>
-      </c>
-      <c r="T88" s="4">
-        <f t="shared" si="19"/>
-        <v>-3.2864017367732464E-4</v>
-      </c>
-      <c r="U88" s="4">
-        <f t="shared" si="20"/>
         <v>-139.52210930120449</v>
       </c>
     </row>
@@ -9400,51 +9455,51 @@
         <v>127.10439</v>
       </c>
       <c r="J89" s="4" t="str">
-        <f>IMDIV(J22,J53)</f>
+        <f t="shared" si="15"/>
         <v>0.999837244380947-6.96285258093127E-06i</v>
       </c>
       <c r="K89" s="4" t="str">
-        <f>IMDIV(K22,K53)</f>
+        <f t="shared" si="15"/>
         <v>-0.561161272596242-0.135374109628846i</v>
       </c>
       <c r="L89" s="4" t="str">
-        <f>IMDIV(L22,L53)</f>
+        <f t="shared" si="15"/>
         <v>0.999844134103527-5.94100918662964E-06i</v>
       </c>
       <c r="M89" s="4" t="str">
-        <f>IMDIV(M22,M53)</f>
+        <f t="shared" si="15"/>
         <v>-0.00674882126193215+0.437367800788996i</v>
       </c>
       <c r="N89" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.4137921888986986E-3</v>
+      </c>
+      <c r="O89" s="4">
+        <f t="shared" si="16"/>
+        <v>-4.7725835261176677</v>
+      </c>
+      <c r="P89" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.3539393410046498E-3</v>
+      </c>
+      <c r="Q89" s="4">
+        <f t="shared" si="18"/>
+        <v>-7.1820299226232684</v>
+      </c>
+      <c r="R89" s="4">
+        <f t="shared" si="23"/>
+        <v>-3.9900700688509714E-4</v>
+      </c>
+      <c r="S89" s="4">
+        <f t="shared" si="19"/>
+        <v>-166.43715034297119</v>
+      </c>
+      <c r="T89" s="4">
+        <f t="shared" si="20"/>
+        <v>-3.4044781664246558E-4</v>
+      </c>
+      <c r="U89" s="4">
         <f t="shared" si="21"/>
-        <v>-1.4137921888986986E-3</v>
-      </c>
-      <c r="O89" s="4">
-        <f t="shared" si="15"/>
-        <v>-4.7725835261176677</v>
-      </c>
-      <c r="P89" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.3539393410046498E-3</v>
-      </c>
-      <c r="Q89" s="4">
-        <f t="shared" si="17"/>
-        <v>-7.1820299226232684</v>
-      </c>
-      <c r="R89" s="4">
-        <f t="shared" si="22"/>
-        <v>-3.9900700688509714E-4</v>
-      </c>
-      <c r="S89" s="4">
-        <f t="shared" si="18"/>
-        <v>-166.43715034297119</v>
-      </c>
-      <c r="T89" s="4">
-        <f t="shared" si="19"/>
-        <v>-3.4044781664246558E-4</v>
-      </c>
-      <c r="U89" s="4">
-        <f t="shared" si="20"/>
         <v>90.884034647865548</v>
       </c>
     </row>
@@ -9453,51 +9508,51 @@
         <v>160.00702200000001</v>
       </c>
       <c r="J90" s="4" t="str">
-        <f>IMDIV(J23,J54)</f>
+        <f t="shared" si="15"/>
         <v>0.999835066976252-8.48880936077973E-06i</v>
       </c>
       <c r="K90" s="4" t="str">
-        <f>IMDIV(K23,K54)</f>
+        <f t="shared" si="15"/>
         <v>0.647191603393935-0.0340237960984154i</v>
       </c>
       <c r="L90" s="4" t="str">
-        <f>IMDIV(L23,L54)</f>
+        <f t="shared" si="15"/>
         <v>0.999844617478848-7.44874297188281E-06i</v>
       </c>
       <c r="M90" s="4" t="str">
-        <f>IMDIV(M23,M54)</f>
+        <f t="shared" si="15"/>
         <v>0.564441566366594-1.63171037950419i</v>
       </c>
       <c r="N90" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.4327078825878731E-3</v>
+      </c>
+      <c r="O90" s="4">
+        <f t="shared" si="16"/>
+        <v>-3.7673562308954516</v>
+      </c>
+      <c r="P90" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.3497400551140742E-3</v>
+      </c>
+      <c r="Q90" s="4">
+        <f t="shared" si="18"/>
+        <v>4.7437261756287636</v>
+      </c>
+      <c r="R90" s="4">
+        <f t="shared" si="23"/>
+        <v>-4.8645318164629899E-4</v>
+      </c>
+      <c r="S90" s="4">
+        <f t="shared" si="19"/>
+        <v>-3.0093514410300308</v>
+      </c>
+      <c r="T90" s="4">
+        <f t="shared" si="20"/>
+        <v>-4.26847859655305E-4</v>
+      </c>
+      <c r="U90" s="4">
         <f t="shared" si="21"/>
-        <v>-1.4327078825878731E-3</v>
-      </c>
-      <c r="O90" s="4">
-        <f t="shared" si="15"/>
-        <v>-3.7673562308954516</v>
-      </c>
-      <c r="P90" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.3497400551140742E-3</v>
-      </c>
-      <c r="Q90" s="4">
-        <f t="shared" si="17"/>
-        <v>4.7437261756287636</v>
-      </c>
-      <c r="R90" s="4">
-        <f t="shared" si="22"/>
-        <v>-4.8645318164629899E-4</v>
-      </c>
-      <c r="S90" s="4">
-        <f t="shared" si="18"/>
-        <v>-3.0093514410300308</v>
-      </c>
-      <c r="T90" s="4">
-        <f t="shared" si="19"/>
-        <v>-4.26847859655305E-4</v>
-      </c>
-      <c r="U90" s="4">
-        <f t="shared" si="20"/>
         <v>-70.918463834491902</v>
       </c>
     </row>
@@ -9506,51 +9561,51 @@
         <v>201.45634899999999</v>
       </c>
       <c r="J91" s="4" t="str">
-        <f>IMDIV(J24,J55)</f>
+        <f t="shared" si="15"/>
         <v>0.999844153874277-0.0000117447218741733i</v>
       </c>
       <c r="K91" s="4" t="str">
-        <f>IMDIV(K24,K55)</f>
+        <f t="shared" si="15"/>
         <v>-4.19420419471721+2.19390119172783i</v>
       </c>
       <c r="L91" s="4" t="str">
-        <f>IMDIV(L24,L55)</f>
+        <f t="shared" si="15"/>
         <v>0.999850100145903-9.92822556501746E-06i</v>
       </c>
       <c r="M91" s="4" t="str">
-        <f>IMDIV(M24,M55)</f>
+        <f t="shared" si="15"/>
         <v>-0.690172831698966+1.55952165130799i</v>
       </c>
       <c r="N91" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.3537671417740416E-3</v>
+      </c>
+      <c r="O91" s="4">
+        <f t="shared" si="16"/>
+        <v>13.503362499839113</v>
+      </c>
+      <c r="P91" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.3021107568139112E-3</v>
+      </c>
+      <c r="Q91" s="4">
+        <f t="shared" si="18"/>
+        <v>4.6366105239142659</v>
+      </c>
+      <c r="R91" s="4">
+        <f t="shared" si="23"/>
+        <v>-6.7302788370233655E-4</v>
+      </c>
+      <c r="S91" s="4">
+        <f t="shared" si="19"/>
+        <v>152.38686741857492</v>
+      </c>
+      <c r="T91" s="4">
+        <f t="shared" si="20"/>
+        <v>-5.6893070554044349E-4</v>
+      </c>
+      <c r="U91" s="4">
         <f t="shared" si="21"/>
-        <v>-1.3537671417740416E-3</v>
-      </c>
-      <c r="O91" s="4">
-        <f t="shared" si="15"/>
-        <v>13.503362499839113</v>
-      </c>
-      <c r="P91" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.3021107568139112E-3</v>
-      </c>
-      <c r="Q91" s="4">
-        <f t="shared" si="17"/>
-        <v>4.6366105239142659</v>
-      </c>
-      <c r="R91" s="4">
-        <f t="shared" si="22"/>
-        <v>-6.7302788370233655E-4</v>
-      </c>
-      <c r="S91" s="4">
-        <f t="shared" si="18"/>
-        <v>152.38686741857492</v>
-      </c>
-      <c r="T91" s="4">
-        <f t="shared" si="19"/>
-        <v>-5.6893070554044349E-4</v>
-      </c>
-      <c r="U91" s="4">
-        <f t="shared" si="20"/>
         <v>113.87198617730586</v>
       </c>
     </row>
@@ -9559,51 +9614,51 @@
         <v>253.58521099999999</v>
       </c>
       <c r="J92" s="4" t="str">
-        <f>IMDIV(J25,J56)</f>
+        <f t="shared" si="15"/>
         <v>0.999856344477252-0.0000123689828915486i</v>
       </c>
       <c r="K92" s="4" t="str">
-        <f>IMDIV(K25,K56)</f>
+        <f t="shared" si="15"/>
         <v>-0.792195383537882-0.466594625998461i</v>
       </c>
       <c r="L92" s="4" t="str">
-        <f>IMDIV(L25,L56)</f>
+        <f t="shared" si="15"/>
         <v>0.999868299577613-0.0000106697871373747i</v>
       </c>
       <c r="M92" s="4" t="str">
-        <f>IMDIV(M25,M56)</f>
+        <f t="shared" si="15"/>
         <v>0.0224331979397233+0.348400107929768i</v>
       </c>
       <c r="N92" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.2478649854036918E-3</v>
+      </c>
+      <c r="O92" s="4">
+        <f t="shared" si="16"/>
+        <v>-0.72997315181692846</v>
+      </c>
+      <c r="P92" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.144010174588519E-3</v>
+      </c>
+      <c r="Q92" s="4">
+        <f t="shared" si="18"/>
+        <v>-9.1404659003679249</v>
+      </c>
+      <c r="R92" s="4">
+        <f t="shared" si="23"/>
+        <v>-7.0879233845300453E-4</v>
+      </c>
+      <c r="S92" s="4">
+        <f t="shared" si="19"/>
+        <v>-149.50236888924255</v>
+      </c>
+      <c r="T92" s="4">
+        <f t="shared" si="20"/>
+        <v>-6.1141429477221262E-4</v>
+      </c>
+      <c r="U92" s="4">
         <f t="shared" si="21"/>
-        <v>-1.2478649854036918E-3</v>
-      </c>
-      <c r="O92" s="4">
-        <f t="shared" si="15"/>
-        <v>-0.72997315181692846</v>
-      </c>
-      <c r="P92" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.144010174588519E-3</v>
-      </c>
-      <c r="Q92" s="4">
-        <f t="shared" si="17"/>
-        <v>-9.1404659003679249</v>
-      </c>
-      <c r="R92" s="4">
-        <f t="shared" si="22"/>
-        <v>-7.0879233845300453E-4</v>
-      </c>
-      <c r="S92" s="4">
-        <f t="shared" si="18"/>
-        <v>-149.50236888924255</v>
-      </c>
-      <c r="T92" s="4">
-        <f t="shared" si="19"/>
-        <v>-6.1141429477221262E-4</v>
-      </c>
-      <c r="U92" s="4">
-        <f t="shared" si="20"/>
         <v>86.315857455459295</v>
       </c>
     </row>
@@ -9612,51 +9667,51 @@
         <v>319.290075</v>
       </c>
       <c r="J93" s="4" t="str">
-        <f>IMDIV(J26,J57)</f>
+        <f t="shared" si="15"/>
         <v>0.99985824394825-0.0000168083181045706i</v>
       </c>
       <c r="K93" s="4" t="str">
-        <f>IMDIV(K26,K57)</f>
+        <f t="shared" si="15"/>
         <v>0.179863567305996-0.625482754746781i</v>
       </c>
       <c r="L93" s="4" t="str">
-        <f>IMDIV(L26,L57)</f>
+        <f t="shared" si="15"/>
         <v>0.999869039841201-0.000014464147995687i</v>
       </c>
       <c r="M93" s="4" t="str">
-        <f>IMDIV(M26,M57)</f>
+        <f t="shared" si="15"/>
         <v>-0.538558467211703-0.691854910140105i</v>
       </c>
       <c r="N93" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.2313634724745004E-3</v>
+      </c>
+      <c r="O93" s="4">
+        <f t="shared" si="16"/>
+        <v>-3.7306498529311254</v>
+      </c>
+      <c r="P93" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.1375790679318701E-3</v>
+      </c>
+      <c r="Q93" s="4">
+        <f t="shared" si="18"/>
+        <v>-1.142383509885843</v>
+      </c>
+      <c r="R93" s="4">
+        <f t="shared" si="23"/>
+        <v>-9.6318222492382916E-4</v>
+      </c>
+      <c r="S93" s="4">
+        <f t="shared" si="19"/>
+        <v>-73.956902915590192</v>
+      </c>
+      <c r="T93" s="4">
+        <f t="shared" si="20"/>
+        <v>-8.2884317978210891E-4</v>
+      </c>
+      <c r="U93" s="4">
         <f t="shared" si="21"/>
-        <v>-1.2313634724745004E-3</v>
-      </c>
-      <c r="O93" s="4">
-        <f t="shared" si="15"/>
-        <v>-3.7306498529311254</v>
-      </c>
-      <c r="P93" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.1375790679318701E-3</v>
-      </c>
-      <c r="Q93" s="4">
-        <f t="shared" si="17"/>
-        <v>-1.142383509885843</v>
-      </c>
-      <c r="R93" s="4">
-        <f t="shared" si="22"/>
-        <v>-9.6318222492382916E-4</v>
-      </c>
-      <c r="S93" s="4">
-        <f t="shared" si="18"/>
-        <v>-73.956902915590192</v>
-      </c>
-      <c r="T93" s="4">
-        <f t="shared" si="19"/>
-        <v>-8.2884317978210891E-4</v>
-      </c>
-      <c r="U93" s="4">
-        <f t="shared" si="20"/>
         <v>-127.89814952074971</v>
       </c>
     </row>
@@ -9665,51 +9720,51 @@
         <v>401.94414</v>
       </c>
       <c r="J94" s="4" t="str">
-        <f>IMDIV(J27,J58)</f>
+        <f t="shared" si="15"/>
         <v>0.999850053782203-0.0000170444232473115i</v>
       </c>
       <c r="K94" s="4" t="str">
-        <f>IMDIV(K27,K58)</f>
+        <f t="shared" si="15"/>
         <v>-0.0628085490648813+0.308324113234354i</v>
       </c>
       <c r="L94" s="4" t="str">
-        <f>IMDIV(L27,L58)</f>
+        <f t="shared" si="15"/>
         <v>0.999861830213744-0.0000151887645687953i</v>
       </c>
       <c r="M94" s="4" t="str">
-        <f>IMDIV(M27,M58)</f>
+        <f t="shared" si="15"/>
         <v>-0.147866231616571-0.00501658320762522i</v>
       </c>
       <c r="N94" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.3025126933328963E-3</v>
+      </c>
+      <c r="O94" s="4">
+        <f t="shared" si="16"/>
+        <v>-10.043267618307956</v>
+      </c>
+      <c r="P94" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.2002094308673603E-3</v>
+      </c>
+      <c r="Q94" s="4">
+        <f t="shared" si="18"/>
+        <v>-16.597624014284179</v>
+      </c>
+      <c r="R94" s="4">
+        <f t="shared" si="23"/>
+        <v>-9.767199716766168E-4</v>
+      </c>
+      <c r="S94" s="4">
+        <f t="shared" si="19"/>
+        <v>101.514149720351</v>
+      </c>
+      <c r="T94" s="4">
+        <f t="shared" si="20"/>
+        <v>-8.7037236490649424E-4</v>
+      </c>
+      <c r="U94" s="4">
         <f t="shared" si="21"/>
-        <v>-1.3025126933328963E-3</v>
-      </c>
-      <c r="O94" s="4">
-        <f t="shared" si="15"/>
-        <v>-10.043267618307956</v>
-      </c>
-      <c r="P94" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.2002094308673603E-3</v>
-      </c>
-      <c r="Q94" s="4">
-        <f t="shared" si="17"/>
-        <v>-16.597624014284179</v>
-      </c>
-      <c r="R94" s="4">
-        <f t="shared" si="22"/>
-        <v>-9.767199716766168E-4</v>
-      </c>
-      <c r="S94" s="4">
-        <f t="shared" si="18"/>
-        <v>101.514149720351</v>
-      </c>
-      <c r="T94" s="4">
-        <f t="shared" si="19"/>
-        <v>-8.7037236490649424E-4</v>
-      </c>
-      <c r="U94" s="4">
-        <f t="shared" si="20"/>
         <v>-178.05690020840714</v>
       </c>
     </row>
@@ -9718,51 +9773,51 @@
         <v>506.01529900000003</v>
       </c>
       <c r="J95" s="4" t="str">
-        <f>IMDIV(J28,J59)</f>
+        <f t="shared" si="15"/>
         <v>0.999857216149203-0.0000295546911667565i</v>
       </c>
       <c r="K95" s="4" t="str">
-        <f>IMDIV(K28,K59)</f>
+        <f t="shared" si="15"/>
         <v>0.0484781293700828+0.293066255547994i</v>
       </c>
       <c r="L95" s="4" t="str">
-        <f>IMDIV(L28,L59)</f>
+        <f t="shared" si="15"/>
         <v>0.999868387845784-0.0000273529505883213i</v>
       </c>
       <c r="M95" s="4" t="str">
-        <f>IMDIV(M28,M59)</f>
+        <f t="shared" si="15"/>
         <v>-1.72622647289633+2.16139307765981i</v>
       </c>
       <c r="N95" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.2402895245992647E-3</v>
+      </c>
+      <c r="O95" s="4">
+        <f t="shared" si="16"/>
+        <v>-10.543445451311362</v>
+      </c>
+      <c r="P95" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.143240630416677E-3</v>
+      </c>
+      <c r="Q95" s="4">
+        <f t="shared" si="18"/>
+        <v>8.8374532660665057</v>
+      </c>
+      <c r="R95" s="4">
+        <f t="shared" si="23"/>
+        <v>-1.6936008870309064E-3</v>
+      </c>
+      <c r="S95" s="4">
+        <f t="shared" si="19"/>
+        <v>80.607359525786833</v>
+      </c>
+      <c r="T95" s="4">
+        <f t="shared" si="20"/>
+        <v>-1.5674149164034345E-3</v>
+      </c>
+      <c r="U95" s="4">
         <f t="shared" si="21"/>
-        <v>-1.2402895245992647E-3</v>
-      </c>
-      <c r="O95" s="4">
-        <f t="shared" si="15"/>
-        <v>-10.543445451311362</v>
-      </c>
-      <c r="P95" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.143240630416677E-3</v>
-      </c>
-      <c r="Q95" s="4">
-        <f t="shared" si="17"/>
-        <v>8.8374532660665057</v>
-      </c>
-      <c r="R95" s="4">
-        <f t="shared" si="22"/>
-        <v>-1.6936008870309064E-3</v>
-      </c>
-      <c r="S95" s="4">
-        <f t="shared" si="18"/>
-        <v>80.607359525786833</v>
-      </c>
-      <c r="T95" s="4">
-        <f t="shared" si="19"/>
-        <v>-1.5674149164034345E-3</v>
-      </c>
-      <c r="U95" s="4">
-        <f t="shared" si="20"/>
         <v>128.61309677031463</v>
       </c>
     </row>
@@ -9771,51 +9826,51 @@
         <v>636.97722999999996</v>
       </c>
       <c r="J96" s="4" t="str">
-        <f>IMDIV(J29,J60)</f>
+        <f t="shared" si="15"/>
         <v>0.999853690287979-0.0000289304180355038i</v>
       </c>
       <c r="K96" s="4" t="str">
-        <f>IMDIV(K29,K60)</f>
+        <f t="shared" si="15"/>
         <v>-0.944927815260961+0.303688509608043i</v>
       </c>
       <c r="L96" s="4" t="str">
-        <f>IMDIV(L29,L60)</f>
+        <f t="shared" si="15"/>
         <v>0.999865507614265-0.000025141143244811i</v>
       </c>
       <c r="M96" s="4" t="str">
-        <f>IMDIV(M29,M60)</f>
+        <f t="shared" si="15"/>
         <v>-0.873173120697588+0.18564541381465i</v>
       </c>
       <c r="N96" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.2709193520738507E-3</v>
+      </c>
+      <c r="O96" s="4">
+        <f t="shared" si="16"/>
+        <v>-6.5129415388004791E-2</v>
+      </c>
+      <c r="P96" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.1682618369467843E-3</v>
+      </c>
+      <c r="Q96" s="4">
+        <f t="shared" si="18"/>
+        <v>-0.98598615574881565</v>
+      </c>
+      <c r="R96" s="4">
+        <f t="shared" si="23"/>
+        <v>-1.6578334096496844E-3</v>
+      </c>
+      <c r="S96" s="4">
+        <f t="shared" si="19"/>
+        <v>162.18321531695761</v>
+      </c>
+      <c r="T96" s="4">
+        <f t="shared" si="20"/>
+        <v>-1.4406751595972137E-3</v>
+      </c>
+      <c r="U96" s="4">
         <f t="shared" si="21"/>
-        <v>-1.2709193520738507E-3</v>
-      </c>
-      <c r="O96" s="4">
-        <f t="shared" si="15"/>
-        <v>-6.5129415388004791E-2</v>
-      </c>
-      <c r="P96" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.1682618369467843E-3</v>
-      </c>
-      <c r="Q96" s="4">
-        <f t="shared" si="17"/>
-        <v>-0.98598615574881565</v>
-      </c>
-      <c r="R96" s="4">
-        <f t="shared" si="22"/>
-        <v>-1.6578334096496844E-3</v>
-      </c>
-      <c r="S96" s="4">
-        <f t="shared" si="18"/>
-        <v>162.18321531695761</v>
-      </c>
-      <c r="T96" s="4">
-        <f t="shared" si="19"/>
-        <v>-1.4406751595972137E-3</v>
-      </c>
-      <c r="U96" s="4">
-        <f t="shared" si="20"/>
         <v>167.99706578352257</v>
       </c>
     </row>
@@ -9824,51 +9879,51 @@
         <v>801.91144499999996</v>
       </c>
       <c r="J97" s="4" t="str">
-        <f>IMDIV(J30,J61)</f>
+        <f t="shared" si="15"/>
         <v>0.999853905694553-0.0000363317855039376i</v>
       </c>
       <c r="K97" s="4" t="str">
-        <f>IMDIV(K30,K61)</f>
+        <f t="shared" si="15"/>
         <v>0.820847610413268+1.14465668812107i</v>
       </c>
       <c r="L97" s="4" t="str">
-        <f>IMDIV(L30,L61)</f>
+        <f t="shared" si="15"/>
         <v>0.999862587524773-0.0000310113817618854i</v>
       </c>
       <c r="M97" s="4" t="str">
-        <f>IMDIV(M30,M61)</f>
+        <f t="shared" si="15"/>
         <v>-0.440471443915085-0.311494086366272i</v>
       </c>
       <c r="N97" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.2690459823785157E-3</v>
+      </c>
+      <c r="O97" s="4">
+        <f t="shared" si="16"/>
+        <v>2.975481763160845</v>
+      </c>
+      <c r="P97" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.1936274287472296E-3</v>
+      </c>
+      <c r="Q97" s="4">
+        <f t="shared" si="18"/>
+        <v>-5.3604185867667713</v>
+      </c>
+      <c r="R97" s="4">
+        <f t="shared" si="23"/>
+        <v>-2.0819621334458656E-3</v>
+      </c>
+      <c r="S97" s="4">
+        <f t="shared" si="19"/>
+        <v>54.355220122434538</v>
+      </c>
+      <c r="T97" s="4">
+        <f t="shared" si="20"/>
+        <v>-1.7770654822218115E-3</v>
+      </c>
+      <c r="U97" s="4">
         <f t="shared" si="21"/>
-        <v>-1.2690459823785157E-3</v>
-      </c>
-      <c r="O97" s="4">
-        <f t="shared" si="15"/>
-        <v>2.975481763160845</v>
-      </c>
-      <c r="P97" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.1936274287472296E-3</v>
-      </c>
-      <c r="Q97" s="4">
-        <f t="shared" si="17"/>
-        <v>-5.3604185867667713</v>
-      </c>
-      <c r="R97" s="4">
-        <f t="shared" si="22"/>
-        <v>-2.0819621334458656E-3</v>
-      </c>
-      <c r="S97" s="4">
-        <f t="shared" si="18"/>
-        <v>54.355220122434538</v>
-      </c>
-      <c r="T97" s="4">
-        <f t="shared" si="19"/>
-        <v>-1.7770654822218115E-3</v>
-      </c>
-      <c r="U97" s="4">
-        <f t="shared" si="20"/>
         <v>-144.73268440203074</v>
       </c>
     </row>
@@ -9877,51 +9932,51 @@
         <v>1009.546788</v>
       </c>
       <c r="J98" s="4" t="str">
-        <f>IMDIV(J31,J62)</f>
+        <f t="shared" si="15"/>
         <v>0.999855335177261-0.0000441178730538819i</v>
       </c>
       <c r="K98" s="4" t="str">
-        <f>IMDIV(K31,K62)</f>
+        <f t="shared" si="15"/>
         <v>-1.25957722369317+1.39224075738156i</v>
       </c>
       <c r="L98" s="4" t="str">
-        <f>IMDIV(L31,L62)</f>
+        <f t="shared" si="15"/>
         <v>0.999867479323995-0.0000385093099683711i</v>
       </c>
       <c r="M98" s="4" t="str">
-        <f>IMDIV(M31,M62)</f>
+        <f t="shared" si="15"/>
         <v>0.271633434803804+0.572548052977831i</v>
       </c>
       <c r="N98" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.2566251268545645E-3</v>
+      </c>
+      <c r="O98" s="4">
+        <f t="shared" si="16"/>
+        <v>5.4714299471425409</v>
+      </c>
+      <c r="P98" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.1511298007511573E-3</v>
+      </c>
+      <c r="Q98" s="4">
+        <f t="shared" si="18"/>
+        <v>-3.962106259909175</v>
+      </c>
+      <c r="R98" s="4">
+        <f t="shared" si="23"/>
+        <v>-2.528133657448309E-3</v>
+      </c>
+      <c r="S98" s="4">
+        <f t="shared" si="19"/>
+        <v>132.1360293292876</v>
+      </c>
+      <c r="T98" s="4">
+        <f t="shared" si="20"/>
+        <v>-2.2067133672049326E-3</v>
+      </c>
+      <c r="U98" s="4">
         <f t="shared" si="21"/>
-        <v>-1.2566251268545645E-3</v>
-      </c>
-      <c r="O98" s="4">
-        <f t="shared" si="15"/>
-        <v>5.4714299471425409</v>
-      </c>
-      <c r="P98" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.1511298007511573E-3</v>
-      </c>
-      <c r="Q98" s="4">
-        <f t="shared" si="17"/>
-        <v>-3.962106259909175</v>
-      </c>
-      <c r="R98" s="4">
-        <f t="shared" si="22"/>
-        <v>-2.528133657448309E-3</v>
-      </c>
-      <c r="S98" s="4">
-        <f t="shared" si="18"/>
-        <v>132.1360293292876</v>
-      </c>
-      <c r="T98" s="4">
-        <f t="shared" si="19"/>
-        <v>-2.2067133672049326E-3</v>
-      </c>
-      <c r="U98" s="4">
-        <f t="shared" si="20"/>
         <v>64.618978203090791</v>
       </c>
     </row>
@@ -9930,51 +9985,51 @@
         <v>1271.06546</v>
       </c>
       <c r="J99" s="4" t="str">
-        <f>IMDIV(J32,J63)</f>
+        <f t="shared" si="15"/>
         <v>0.999865188806063-0.0000598708202099452i</v>
       </c>
       <c r="K99" s="4" t="str">
-        <f>IMDIV(K32,K63)</f>
+        <f t="shared" si="15"/>
         <v>-1.14680055200298-0.672709813856939i</v>
       </c>
       <c r="L99" s="4" t="str">
-        <f>IMDIV(L32,L63)</f>
+        <f t="shared" si="15"/>
         <v>0.999874370158014-0.0000528094744369557i</v>
       </c>
       <c r="M99" s="4" t="str">
-        <f>IMDIV(M32,M63)</f>
+        <f t="shared" si="15"/>
         <v>0.00900576906225159-0.115211817870034i</v>
       </c>
       <c r="N99" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.1710185169889519E-3</v>
+      </c>
+      <c r="O99" s="4">
+        <f t="shared" si="16"/>
+        <v>2.4740610501557705</v>
+      </c>
+      <c r="P99" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.0912633777326111E-3</v>
+      </c>
+      <c r="Q99" s="4">
+        <f t="shared" si="18"/>
+        <v>-18.743604374933344</v>
+      </c>
+      <c r="R99" s="4">
+        <f t="shared" si="23"/>
+        <v>-3.4308078212151459E-3</v>
+      </c>
+      <c r="S99" s="4">
+        <f t="shared" si="19"/>
+        <v>-149.60424005283531</v>
+      </c>
+      <c r="T99" s="4">
+        <f t="shared" si="20"/>
+        <v>-3.026140174239994E-3</v>
+      </c>
+      <c r="U99" s="4">
         <f t="shared" si="21"/>
-        <v>-1.1710185169889519E-3</v>
-      </c>
-      <c r="O99" s="4">
-        <f t="shared" si="15"/>
-        <v>2.4740610501557705</v>
-      </c>
-      <c r="P99" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.0912633777326111E-3</v>
-      </c>
-      <c r="Q99" s="4">
-        <f t="shared" si="17"/>
-        <v>-18.743604374933344</v>
-      </c>
-      <c r="R99" s="4">
-        <f t="shared" si="22"/>
-        <v>-3.4308078212151459E-3</v>
-      </c>
-      <c r="S99" s="4">
-        <f t="shared" si="18"/>
-        <v>-149.60424005283531</v>
-      </c>
-      <c r="T99" s="4">
-        <f t="shared" si="19"/>
-        <v>-3.026140174239994E-3</v>
-      </c>
-      <c r="U99" s="4">
-        <f t="shared" si="20"/>
         <v>-85.530445714190037</v>
       </c>
     </row>
@@ -9983,51 +10038,51 @@
         <v>1600.019278</v>
       </c>
       <c r="J100" s="4" t="str">
-        <f>IMDIV(J33,J64)</f>
+        <f t="shared" si="15"/>
         <v>0.999856769315902-0.0000765634419466034i</v>
       </c>
       <c r="K100" s="4" t="str">
-        <f>IMDIV(K33,K64)</f>
+        <f t="shared" si="15"/>
         <v>0.856973533073068+0.747052353315737i</v>
       </c>
       <c r="L100" s="4" t="str">
-        <f>IMDIV(L33,L64)</f>
+        <f t="shared" si="15"/>
         <v>0.999867792485655-0.0000682620823012735i</v>
       </c>
       <c r="M100" s="4" t="str">
-        <f>IMDIV(M33,M64)</f>
+        <f t="shared" si="15"/>
         <v>0.547348050117526+0.0310092516072573i</v>
       </c>
       <c r="N100" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.2441495535406384E-3</v>
+      </c>
+      <c r="O100" s="4">
+        <f t="shared" si="16"/>
+        <v>1.1142747892670199</v>
+      </c>
+      <c r="P100" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.1483955529717942E-3</v>
+      </c>
+      <c r="Q100" s="4">
+        <f t="shared" si="18"/>
+        <v>-5.2208115561365274</v>
+      </c>
+      <c r="R100" s="4">
+        <f t="shared" si="23"/>
+        <v>-4.3873904889022656E-3</v>
+      </c>
+      <c r="S100" s="4">
+        <f t="shared" si="19"/>
+        <v>41.079746188860966</v>
+      </c>
+      <c r="T100" s="4">
+        <f t="shared" si="20"/>
+        <v>-3.9116463596033267E-3</v>
+      </c>
+      <c r="U100" s="4">
         <f t="shared" si="21"/>
-        <v>-1.2441495535406384E-3</v>
-      </c>
-      <c r="O100" s="4">
-        <f t="shared" si="15"/>
-        <v>1.1142747892670199</v>
-      </c>
-      <c r="P100" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.1483955529717942E-3</v>
-      </c>
-      <c r="Q100" s="4">
-        <f t="shared" si="17"/>
-        <v>-5.2208115561365274</v>
-      </c>
-      <c r="R100" s="4">
-        <f t="shared" si="22"/>
-        <v>-4.3873904889022656E-3</v>
-      </c>
-      <c r="S100" s="4">
-        <f t="shared" si="18"/>
-        <v>41.079746188860966</v>
-      </c>
-      <c r="T100" s="4">
-        <f t="shared" si="19"/>
-        <v>-3.9116463596033267E-3</v>
-      </c>
-      <c r="U100" s="4">
-        <f t="shared" si="20"/>
         <v>3.24254748655179</v>
       </c>
     </row>
@@ -10036,51 +10091,51 @@
         <v>2014.3138919999999</v>
       </c>
       <c r="J101" s="4" t="str">
-        <f>IMDIV(J34,J65)</f>
+        <f t="shared" si="15"/>
         <v>0.999868335238889-0.000087528756223352i</v>
       </c>
       <c r="K101" s="4" t="str">
-        <f>IMDIV(K34,K65)</f>
+        <f t="shared" si="15"/>
         <v>1.10018023304069+0.388131300213762i</v>
       </c>
       <c r="L101" s="4" t="str">
-        <f>IMDIV(L34,L65)</f>
+        <f t="shared" si="15"/>
         <v>0.999881163853038-0.000077063081353247i</v>
       </c>
       <c r="M101" s="4" t="str">
-        <f>IMDIV(M34,M65)</f>
+        <f t="shared" si="15"/>
         <v>-0.197838720924812+0.262013525247772i</v>
       </c>
       <c r="N101" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.1436675971426542E-3</v>
+      </c>
+      <c r="O101" s="4">
+        <f t="shared" si="16"/>
+        <v>1.3387167120786598</v>
+      </c>
+      <c r="P101" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.032233195922425E-3</v>
+      </c>
+      <c r="Q101" s="4">
+        <f t="shared" si="18"/>
+        <v>-9.6741650420547654</v>
+      </c>
+      <c r="R101" s="4">
+        <f t="shared" si="23"/>
+        <v>-5.0156886942706895E-3</v>
+      </c>
+      <c r="S101" s="4">
+        <f t="shared" si="19"/>
+        <v>19.432272670255237</v>
+      </c>
+      <c r="T101" s="4">
+        <f t="shared" si="20"/>
+        <v>-4.4159140792862017E-3</v>
+      </c>
+      <c r="U101" s="4">
         <f t="shared" si="21"/>
-        <v>-1.1436675971426542E-3</v>
-      </c>
-      <c r="O101" s="4">
-        <f t="shared" si="15"/>
-        <v>1.3387167120786598</v>
-      </c>
-      <c r="P101" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.032233195922425E-3</v>
-      </c>
-      <c r="Q101" s="4">
-        <f t="shared" si="17"/>
-        <v>-9.6741650420547654</v>
-      </c>
-      <c r="R101" s="4">
-        <f t="shared" si="22"/>
-        <v>-5.0156886942706895E-3</v>
-      </c>
-      <c r="S101" s="4">
-        <f t="shared" si="18"/>
-        <v>19.432272670255237</v>
-      </c>
-      <c r="T101" s="4">
-        <f t="shared" si="19"/>
-        <v>-4.4159140792862017E-3</v>
-      </c>
-      <c r="U101" s="4">
-        <f t="shared" si="20"/>
         <v>127.05538245872529</v>
       </c>
     </row>
@@ -10089,51 +10144,51 @@
         <v>2536.1076779999999</v>
       </c>
       <c r="J102" s="4" t="str">
-        <f>IMDIV(J35,J66)</f>
+        <f t="shared" si="15"/>
         <v>0.999857691066968-0.000109387919487617i</v>
       </c>
       <c r="K102" s="4" t="str">
-        <f>IMDIV(K35,K66)</f>
+        <f t="shared" si="15"/>
         <v>0.306693905024399-0.252902734281646i</v>
       </c>
       <c r="L102" s="4" t="str">
-        <f>IMDIV(L35,L66)</f>
+        <f t="shared" si="15"/>
         <v>0.999868424020532-0.0000968309852225643i</v>
       </c>
       <c r="M102" s="4" t="str">
-        <f>IMDIV(M35,M66)</f>
+        <f t="shared" si="15"/>
         <v>0.293532851471857-0.298674905077673i</v>
       </c>
       <c r="N102" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.2361156665220707E-3</v>
+      </c>
+      <c r="O102" s="4">
+        <f t="shared" si="16"/>
+        <v>-8.0128534704212591</v>
+      </c>
+      <c r="P102" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.1428888981611788E-3</v>
+      </c>
+      <c r="Q102" s="4">
+        <f t="shared" si="18"/>
+        <v>-7.5604907190318311</v>
+      </c>
+      <c r="R102" s="4">
+        <f t="shared" si="23"/>
+        <v>-6.2683581347099592E-3</v>
+      </c>
+      <c r="S102" s="4">
+        <f t="shared" si="19"/>
+        <v>-39.509318772078942</v>
+      </c>
+      <c r="T102" s="4">
+        <f t="shared" si="20"/>
+        <v>-5.5487368424870604E-3</v>
+      </c>
+      <c r="U102" s="4">
         <f t="shared" si="21"/>
-        <v>-1.2361156665220707E-3</v>
-      </c>
-      <c r="O102" s="4">
-        <f t="shared" si="15"/>
-        <v>-8.0128534704212591</v>
-      </c>
-      <c r="P102" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.1428888981611788E-3</v>
-      </c>
-      <c r="Q102" s="4">
-        <f t="shared" si="17"/>
-        <v>-7.5604907190318311</v>
-      </c>
-      <c r="R102" s="4">
-        <f t="shared" si="22"/>
-        <v>-6.2683581347099592E-3</v>
-      </c>
-      <c r="S102" s="4">
-        <f t="shared" si="18"/>
-        <v>-39.509318772078942</v>
-      </c>
-      <c r="T102" s="4">
-        <f t="shared" si="19"/>
-        <v>-5.5487368424870604E-3</v>
-      </c>
-      <c r="U102" s="4">
-        <f t="shared" si="20"/>
         <v>-45.497478398042183</v>
       </c>
     </row>
@@ -10142,51 +10197,51 @@
         <v>3192.5215979999998</v>
       </c>
       <c r="J103" s="4" t="str">
-        <f>IMDIV(J36,J67)</f>
+        <f t="shared" si="15"/>
         <v>0.999873816451977-0.000115284158449535i</v>
       </c>
       <c r="K103" s="4" t="str">
-        <f>IMDIV(K36,K67)</f>
+        <f t="shared" si="15"/>
         <v>-1.08674899157468+1.47219001848447i</v>
       </c>
       <c r="L103" s="4" t="str">
-        <f>IMDIV(L36,L67)</f>
+        <f t="shared" si="15"/>
         <v>0.999883961837353-0.000100065347067376i</v>
       </c>
       <c r="M103" s="4" t="str">
-        <f>IMDIV(M36,M67)</f>
+        <f t="shared" si="15"/>
         <v>1.18740016202776+2.16368478408872i</v>
       </c>
       <c r="N103" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.0960277934979419E-3</v>
+      </c>
+      <c r="O103" s="4">
+        <f t="shared" si="16"/>
+        <v>5.2483302987750013</v>
+      </c>
+      <c r="P103" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.0079096598832828E-3</v>
+      </c>
+      <c r="Q103" s="4">
+        <f t="shared" si="18"/>
+        <v>7.8472075433297945</v>
+      </c>
+      <c r="R103" s="4">
+        <f t="shared" si="23"/>
+        <v>-6.6061292794371736E-3</v>
+      </c>
+      <c r="S103" s="4">
+        <f t="shared" si="19"/>
+        <v>126.43419737673742</v>
+      </c>
+      <c r="T103" s="4">
+        <f t="shared" si="20"/>
+        <v>-5.7339874046950156E-3</v>
+      </c>
+      <c r="U103" s="4">
         <f t="shared" si="21"/>
-        <v>-1.0960277934979419E-3</v>
-      </c>
-      <c r="O103" s="4">
-        <f t="shared" si="15"/>
-        <v>5.2483302987750013</v>
-      </c>
-      <c r="P103" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.0079096598832828E-3</v>
-      </c>
-      <c r="Q103" s="4">
-        <f t="shared" si="17"/>
-        <v>7.8472075433297945</v>
-      </c>
-      <c r="R103" s="4">
-        <f t="shared" si="22"/>
-        <v>-6.6061292794371736E-3</v>
-      </c>
-      <c r="S103" s="4">
-        <f t="shared" si="18"/>
-        <v>126.43419737673742</v>
-      </c>
-      <c r="T103" s="4">
-        <f t="shared" si="19"/>
-        <v>-5.7339874046950156E-3</v>
-      </c>
-      <c r="U103" s="4">
-        <f t="shared" si="20"/>
         <v>61.242631409213438</v>
       </c>
     </row>
@@ -10195,51 +10250,51 @@
         <v>4019.4603149999998</v>
       </c>
       <c r="J104" s="4" t="str">
-        <f>IMDIV(J37,J68)</f>
+        <f t="shared" si="15"/>
         <v>0.99987254801479-0.000129923593606289i</v>
       </c>
       <c r="K104" s="4" t="str">
-        <f>IMDIV(K37,K68)</f>
+        <f t="shared" si="15"/>
         <v>0.17418922028964+0.247451708601555i</v>
       </c>
       <c r="L104" s="4" t="str">
-        <f>IMDIV(L37,L68)</f>
+        <f t="shared" si="15"/>
         <v>0.999890702823637-0.000112950559907869i</v>
       </c>
       <c r="M104" s="4" t="str">
-        <f>IMDIV(M37,M68)</f>
+        <f t="shared" si="15"/>
         <v>0.563809931973806+0.570064491912739i</v>
       </c>
       <c r="N104" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.1070311023078756E-3</v>
+      </c>
+      <c r="O104" s="4">
+        <f t="shared" si="16"/>
+        <v>-10.3822671228723</v>
+      </c>
+      <c r="P104" s="4">
+        <f t="shared" si="17"/>
+        <v>-9.493396770265223E-4</v>
+      </c>
+      <c r="Q104" s="4">
+        <f t="shared" si="18"/>
+        <v>-1.9188686287158121</v>
+      </c>
+      <c r="R104" s="4">
+        <f t="shared" si="23"/>
+        <v>-7.4450224138034714E-3</v>
+      </c>
+      <c r="S104" s="4">
+        <f t="shared" si="19"/>
+        <v>54.857052770404792</v>
+      </c>
+      <c r="T104" s="4">
+        <f t="shared" si="20"/>
+        <v>-6.4722977527022453E-3</v>
+      </c>
+      <c r="U104" s="4">
         <f t="shared" si="21"/>
-        <v>-1.1070311023078756E-3</v>
-      </c>
-      <c r="O104" s="4">
-        <f t="shared" si="15"/>
-        <v>-10.3822671228723</v>
-      </c>
-      <c r="P104" s="4">
-        <f t="shared" si="16"/>
-        <v>-9.493396770265223E-4</v>
-      </c>
-      <c r="Q104" s="4">
-        <f t="shared" si="17"/>
-        <v>-1.9188686287158121</v>
-      </c>
-      <c r="R104" s="4">
-        <f t="shared" si="22"/>
-        <v>-7.4450224138034714E-3</v>
-      </c>
-      <c r="S104" s="4">
-        <f t="shared" si="18"/>
-        <v>54.857052770404792</v>
-      </c>
-      <c r="T104" s="4">
-        <f t="shared" si="19"/>
-        <v>-6.4722977527022453E-3</v>
-      </c>
-      <c r="U104" s="4">
-        <f t="shared" si="20"/>
         <v>45.316045802856813</v>
       </c>
     </row>
@@ -10248,51 +10303,51 @@
         <v>5059.7908310000003</v>
       </c>
       <c r="J105" s="4" t="str">
-        <f>IMDIV(J38,J69)</f>
+        <f t="shared" si="15"/>
         <v>0.999862915368008-0.000178332410205718i</v>
       </c>
       <c r="K105" s="4" t="str">
-        <f>IMDIV(K38,K69)</f>
+        <f t="shared" si="15"/>
         <v>-0.756196780748331+0.0301330299567231i</v>
       </c>
       <c r="L105" s="4" t="str">
-        <f>IMDIV(L38,L69)</f>
+        <f t="shared" si="15"/>
         <v>0.999884062640059-0.000158167949323925i</v>
       </c>
       <c r="M105" s="4" t="str">
-        <f>IMDIV(M38,M69)</f>
+        <f t="shared" si="15"/>
         <v>-2.20680181357035+3.74745932656229i</v>
       </c>
       <c r="N105" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.1906454513365772E-3</v>
+      </c>
+      <c r="O105" s="4">
+        <f t="shared" si="16"/>
+        <v>-2.4204129379586421</v>
+      </c>
+      <c r="P105" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.0069688203748503E-3</v>
+      </c>
+      <c r="Q105" s="4">
+        <f t="shared" si="18"/>
+        <v>12.767701965103534</v>
+      </c>
+      <c r="R105" s="4">
+        <f t="shared" si="23"/>
+        <v>-1.0219095227746357E-2</v>
+      </c>
+      <c r="S105" s="4">
+        <f t="shared" si="19"/>
+        <v>177.71807744344252</v>
+      </c>
+      <c r="T105" s="4">
+        <f t="shared" si="20"/>
+        <v>-9.0634066623516748E-3</v>
+      </c>
+      <c r="U105" s="4">
         <f t="shared" si="21"/>
-        <v>-1.1906454513365772E-3</v>
-      </c>
-      <c r="O105" s="4">
-        <f t="shared" si="15"/>
-        <v>-2.4204129379586421</v>
-      </c>
-      <c r="P105" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.0069688203748503E-3</v>
-      </c>
-      <c r="Q105" s="4">
-        <f t="shared" si="17"/>
-        <v>12.767701965103534</v>
-      </c>
-      <c r="R105" s="4">
-        <f t="shared" si="22"/>
-        <v>-1.0219095227746357E-2</v>
-      </c>
-      <c r="S105" s="4">
-        <f t="shared" si="18"/>
-        <v>177.71807744344252</v>
-      </c>
-      <c r="T105" s="4">
-        <f t="shared" si="19"/>
-        <v>-9.0634066623516748E-3</v>
-      </c>
-      <c r="U105" s="4">
-        <f t="shared" si="20"/>
         <v>120.4929571474012</v>
       </c>
     </row>
@@ -10301,51 +10356,51 @@
         <v>6369.7354210000003</v>
       </c>
       <c r="J106" s="4" t="str">
-        <f>IMDIV(J39,J70)</f>
+        <f t="shared" si="15"/>
         <v>0.999851361145337-0.000181262103943853i</v>
       </c>
       <c r="K106" s="4" t="str">
-        <f>IMDIV(K39,K70)</f>
+        <f t="shared" si="15"/>
         <v>1.30740568459+0.84613395851928i</v>
       </c>
       <c r="L106" s="4" t="str">
-        <f>IMDIV(L39,L70)</f>
+        <f t="shared" si="15"/>
         <v>0.999878251146311-0.000159060488463645i</v>
       </c>
       <c r="M106" s="4" t="str">
-        <f>IMDIV(M39,M70)</f>
+        <f t="shared" si="15"/>
         <v>0.978818564381325-0.309232686041097i</v>
       </c>
       <c r="N106" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.2910139139264969E-3</v>
+      </c>
+      <c r="O106" s="4">
+        <f t="shared" si="16"/>
+        <v>3.8475692509761434</v>
+      </c>
+      <c r="P106" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.057451582159117E-3</v>
+      </c>
+      <c r="Q106" s="4">
+        <f t="shared" si="18"/>
+        <v>0.227213638163276</v>
+      </c>
+      <c r="R106" s="4">
+        <f t="shared" si="23"/>
+        <v>-1.0387097354122172E-2</v>
+      </c>
+      <c r="S106" s="4">
+        <f t="shared" si="19"/>
+        <v>32.91035731816735</v>
+      </c>
+      <c r="T106" s="4">
+        <f t="shared" si="20"/>
+        <v>-9.1146042920039784E-3</v>
+      </c>
+      <c r="U106" s="4">
         <f t="shared" si="21"/>
-        <v>-1.2910139139264969E-3</v>
-      </c>
-      <c r="O106" s="4">
-        <f t="shared" si="15"/>
-        <v>3.8475692509761434</v>
-      </c>
-      <c r="P106" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.057451582159117E-3</v>
-      </c>
-      <c r="Q106" s="4">
-        <f t="shared" si="17"/>
-        <v>0.227213638163276</v>
-      </c>
-      <c r="R106" s="4">
-        <f t="shared" si="22"/>
-        <v>-1.0387097354122172E-2</v>
-      </c>
-      <c r="S106" s="4">
-        <f t="shared" si="18"/>
-        <v>32.91035731816735</v>
-      </c>
-      <c r="T106" s="4">
-        <f t="shared" si="19"/>
-        <v>-9.1146042920039784E-3</v>
-      </c>
-      <c r="U106" s="4">
-        <f t="shared" si="20"/>
         <v>-17.532598766607091</v>
       </c>
     </row>
@@ -10354,51 +10409,51 @@
         <v>8019.2636849999999</v>
       </c>
       <c r="J107" s="4" t="str">
-        <f>IMDIV(J40,J71)</f>
+        <f t="shared" si="15"/>
         <v>0.999834744047229-0.000266414695529749i</v>
       </c>
       <c r="K107" s="4" t="str">
-        <f>IMDIV(K40,K71)</f>
+        <f t="shared" si="15"/>
         <v>0.887348806274034+0.405007523930006i</v>
       </c>
       <c r="L107" s="4" t="str">
-        <f>IMDIV(L40,L71)</f>
+        <f t="shared" si="15"/>
         <v>0.999873107192835-0.000242424307009639i</v>
       </c>
       <c r="M107" s="4" t="str">
-        <f>IMDIV(M40,M71)</f>
+        <f t="shared" si="15"/>
         <v>1.0961349929718-0.576338960723527i</v>
       </c>
       <c r="N107" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.4352052344753607E-3</v>
+      </c>
+      <c r="O107" s="4">
+        <f t="shared" si="16"/>
+        <v>-0.21628180608483941</v>
+      </c>
+      <c r="P107" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.1019915563080785E-3</v>
+      </c>
+      <c r="Q107" s="4">
+        <f t="shared" si="18"/>
+        <v>1.8573433521936678</v>
+      </c>
+      <c r="R107" s="4">
+        <f t="shared" si="23"/>
+        <v>-1.5266960248919671E-2</v>
+      </c>
+      <c r="S107" s="4">
+        <f t="shared" si="19"/>
+        <v>24.533106509482195</v>
+      </c>
+      <c r="T107" s="4">
+        <f t="shared" si="20"/>
+        <v>-1.3891652121600035E-2</v>
+      </c>
+      <c r="U107" s="4">
         <f t="shared" si="21"/>
-        <v>-1.4352052344753607E-3</v>
-      </c>
-      <c r="O107" s="4">
-        <f t="shared" si="15"/>
-        <v>-0.21628180608483941</v>
-      </c>
-      <c r="P107" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.1019915563080785E-3</v>
-      </c>
-      <c r="Q107" s="4">
-        <f t="shared" si="17"/>
-        <v>1.8573433521936678</v>
-      </c>
-      <c r="R107" s="4">
-        <f t="shared" si="22"/>
-        <v>-1.5266960248919671E-2</v>
-      </c>
-      <c r="S107" s="4">
-        <f t="shared" si="18"/>
-        <v>24.533106509482195</v>
-      </c>
-      <c r="T107" s="4">
-        <f t="shared" si="19"/>
-        <v>-1.3891652121600035E-2</v>
-      </c>
-      <c r="U107" s="4">
-        <f t="shared" si="20"/>
         <v>-27.735032536970039</v>
       </c>
     </row>
@@ -10407,51 +10462,51 @@
         <v>10096.471541000001</v>
       </c>
       <c r="J108" s="4" t="str">
-        <f>IMDIV(J41,J72)</f>
+        <f t="shared" si="15"/>
         <v>0.999844725317202-0.000346635695128587i</v>
       </c>
       <c r="K108" s="4" t="str">
-        <f>IMDIV(K41,K72)</f>
+        <f t="shared" si="15"/>
         <v>2.11042304303399-1.23226127304343i</v>
       </c>
       <c r="L108" s="4" t="str">
-        <f>IMDIV(L41,L72)</f>
+        <f t="shared" si="15"/>
         <v>0.999882553213432-0.000324579442078945i</v>
       </c>
       <c r="M108" s="4" t="str">
-        <f>IMDIV(M41,M72)</f>
+        <f t="shared" si="15"/>
         <v>-2.02273065832211-0.433551872330256i</v>
       </c>
       <c r="N108" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.3482814843306966E-3</v>
+      </c>
+      <c r="O108" s="4">
+        <f t="shared" si="16"/>
+        <v>7.7614548839795887</v>
+      </c>
+      <c r="P108" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.0197320920681825E-3</v>
+      </c>
+      <c r="Q108" s="4">
+        <f t="shared" si="18"/>
+        <v>6.3138354626692017</v>
+      </c>
+      <c r="R108" s="4">
+        <f t="shared" si="23"/>
+        <v>-1.986384591611301E-2</v>
+      </c>
+      <c r="S108" s="4">
+        <f t="shared" si="19"/>
+        <v>-30.280357259480731</v>
+      </c>
+      <c r="T108" s="4">
+        <f t="shared" si="20"/>
+        <v>-1.8599215912745728E-2</v>
+      </c>
+      <c r="U108" s="4">
         <f t="shared" si="21"/>
-        <v>-1.3482814843306966E-3</v>
-      </c>
-      <c r="O108" s="4">
-        <f t="shared" si="15"/>
-        <v>7.7614548839795887</v>
-      </c>
-      <c r="P108" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.0197320920681825E-3</v>
-      </c>
-      <c r="Q108" s="4">
-        <f t="shared" si="17"/>
-        <v>6.3138354626692017</v>
-      </c>
-      <c r="R108" s="4">
-        <f t="shared" si="22"/>
-        <v>-1.986384591611301E-2</v>
-      </c>
-      <c r="S108" s="4">
-        <f t="shared" si="18"/>
-        <v>-30.280357259480731</v>
-      </c>
-      <c r="T108" s="4">
-        <f t="shared" si="19"/>
-        <v>-1.8599215912745728E-2</v>
-      </c>
-      <c r="U108" s="4">
-        <f t="shared" si="20"/>
         <v>-167.90227504141686</v>
       </c>
     </row>
@@ -10460,51 +10515,51 @@
         <v>12710.556156000001</v>
       </c>
       <c r="J109" s="4" t="str">
-        <f>IMDIV(J42,J73)</f>
+        <f t="shared" si="15"/>
         <v>0.999826809207763-0.000464329337813341i</v>
       </c>
       <c r="K109" s="4" t="str">
-        <f>IMDIV(K42,K73)</f>
+        <f t="shared" si="15"/>
         <v>-2.0398908668495+1.95609048068709i</v>
       </c>
       <c r="L109" s="4" t="str">
-        <f>IMDIV(L42,L73)</f>
+        <f t="shared" si="15"/>
         <v>0.999872252709156-0.000444838922855464i</v>
       </c>
       <c r="M109" s="4" t="str">
-        <f>IMDIV(M42,M73)</f>
+        <f t="shared" si="15"/>
         <v>-0.155509743809506+0.837345855711766i</v>
       </c>
       <c r="N109" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.5035097188424136E-3</v>
+      </c>
+      <c r="O109" s="4">
+        <f t="shared" si="16"/>
+        <v>9.0240786533751169</v>
+      </c>
+      <c r="P109" s="4">
+        <f t="shared" si="17"/>
+        <v>-1.1088101413061517E-3</v>
+      </c>
+      <c r="Q109" s="4">
+        <f t="shared" si="18"/>
+        <v>-1.3946354373627847</v>
+      </c>
+      <c r="R109" s="4">
+        <f t="shared" si="23"/>
+        <v>-2.660871783310426E-2</v>
+      </c>
+      <c r="S109" s="4">
+        <f t="shared" si="19"/>
+        <v>136.20138317642079</v>
+      </c>
+      <c r="T109" s="4">
+        <f t="shared" si="20"/>
+        <v>-2.5490647522334531E-2</v>
+      </c>
+      <c r="U109" s="4">
         <f t="shared" si="21"/>
-        <v>-1.5035097188424136E-3</v>
-      </c>
-      <c r="O109" s="4">
-        <f t="shared" si="15"/>
-        <v>9.0240786533751169</v>
-      </c>
-      <c r="P109" s="4">
-        <f t="shared" si="16"/>
-        <v>-1.1088101413061517E-3</v>
-      </c>
-      <c r="Q109" s="4">
-        <f t="shared" si="17"/>
-        <v>-1.3946354373627847</v>
-      </c>
-      <c r="R109" s="4">
-        <f t="shared" si="22"/>
-        <v>-2.660871783310426E-2</v>
-      </c>
-      <c r="S109" s="4">
-        <f t="shared" si="18"/>
-        <v>136.20138317642079</v>
-      </c>
-      <c r="T109" s="4">
-        <f t="shared" si="19"/>
-        <v>-2.5490647522334531E-2</v>
-      </c>
-      <c r="U109" s="4">
-        <f t="shared" si="20"/>
         <v>100.52096001385756</v>
       </c>
     </row>
@@ -10513,51 +10568,51 @@
         <v>16000.960204000001</v>
       </c>
       <c r="J110" s="4" t="str">
-        <f>IMDIV(J43,J74)</f>
+        <f t="shared" si="15"/>
         <v>0.999838043007382-0.000477960443480944i</v>
       </c>
       <c r="K110" s="4" t="str">
-        <f>IMDIV(K43,K74)</f>
+        <f t="shared" si="15"/>
         <v>2.63138465464156+0.909311802769427i</v>
       </c>
       <c r="L110" s="4" t="str">
-        <f>IMDIV(L43,L74)</f>
+        <f t="shared" si="15"/>
         <v>0.999887790000413-0.000463399680672354i</v>
       </c>
       <c r="M110" s="4" t="str">
-        <f>IMDIV(M43,M74)</f>
+        <f t="shared" si="15"/>
         <v>0.43686788781869-0.96097605047088i</v>
       </c>
       <c r="N110" s="4">
+        <f t="shared" si="22"/>
+        <v>-1.4058620415229855E-3</v>
+      </c>
+      <c r="O110" s="4">
+        <f t="shared" si="16"/>
+        <v>8.8935959460405467</v>
+      </c>
+      <c r="P110" s="4">
+        <f t="shared" si="17"/>
+        <v>-9.7376554916999954E-4</v>
+      </c>
+      <c r="Q110" s="4">
+        <f t="shared" si="18"/>
+        <v>0.47013246329529579</v>
+      </c>
+      <c r="R110" s="4">
+        <f t="shared" si="23"/>
+        <v>-2.738955002879391E-2</v>
+      </c>
+      <c r="S110" s="4">
+        <f t="shared" si="19"/>
+        <v>19.063306910155042</v>
+      </c>
+      <c r="T110" s="4">
+        <f t="shared" si="20"/>
+        <v>-2.6553823633845564E-2</v>
+      </c>
+      <c r="U110" s="4">
         <f t="shared" si="21"/>
-        <v>-1.4058620415229855E-3</v>
-      </c>
-      <c r="O110" s="4">
-        <f t="shared" si="15"/>
-        <v>8.8935959460405467</v>
-      </c>
-      <c r="P110" s="4">
-        <f t="shared" si="16"/>
-        <v>-9.7376554916999954E-4</v>
-      </c>
-      <c r="Q110" s="4">
-        <f t="shared" si="17"/>
-        <v>0.47013246329529579</v>
-      </c>
-      <c r="R110" s="4">
-        <f t="shared" si="22"/>
-        <v>-2.738955002879391E-2</v>
-      </c>
-      <c r="S110" s="4">
-        <f t="shared" si="18"/>
-        <v>19.063306910155042</v>
-      </c>
-      <c r="T110" s="4">
-        <f t="shared" si="19"/>
-        <v>-2.6553823633845564E-2</v>
-      </c>
-      <c r="U110" s="4">
-        <f t="shared" si="20"/>
         <v>-65.553051241406976</v>
       </c>
     </row>

</xml_diff>